<commit_message>
feat: implement modern threaded comments with stable relationships and standards compliance
</commit_message>
<xml_diff>
--- a/Tests/Fixtures/thread_comments.xlsx
+++ b/Tests/Fixtures/thread_comments.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/2342184/programs/OpenXLSX/Tests/Fixtures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D879BB4-8C31-734F-9A02-992F49050029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0613E7-CE90-4F40-B54D-D0184FC374C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3220" yWindow="2160" windowWidth="28100" windowHeight="17360" xr2:uid="{0C52AA12-D58F-7D4C-86DF-F1B519ACB25B}"/>
   </bookViews>
@@ -39,6 +39,8 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={62B73EE7-EA2E-CD42-ABDF-55112CEEA85C}</author>
+    <author>tc={7DB408AD-9FCB-6047-8FBF-78F298A51E18}</author>
+    <author>tc={5139E8D2-ECA7-044F-8352-0F7F0BD80678}</author>
   </authors>
   <commentList>
     <comment ref="B2" authorId="0" shapeId="0" xr:uid="{62B73EE7-EA2E-CD42-ABDF-55112CEEA85C}">
@@ -51,14 +53,44 @@
     I'm fine.</t>
       </text>
     </comment>
+    <comment ref="C4" authorId="1" shapeId="0" xr:uid="{7DB408AD-9FCB-6047-8FBF-78F298A51E18}">
+      <text>
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
+    好的
+答复:
+    不错
+答复:
+    很好</t>
+      </text>
+    </comment>
+    <comment ref="C8" authorId="2" shapeId="0" xr:uid="{5139E8D2-ECA7-044F-8352-0F7F0BD80678}">
+      <text>
+        <t>[线程批注]
+你的Excel版本可读取此线程批注; 但如果在更新版本的Excel中打开文件，则对批注所作的任何改动都将被删除。了解详细信息: https://go.microsoft.com/fwlink/?linkid=870924
+注释:
+    world 
+答复:
+    这是回复</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Hello</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>World</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>这是多个批注</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -462,20 +494,47 @@
   <threadedComment ref="B2" dT="2026-04-02T14:25:05.79" personId="{3593DA02-0F55-9F40-9BF5-CE90CCFAECBC}" id="{77210FAD-397A-8747-8770-9D6D3FD2FA5C}" parentId="{62B73EE7-EA2E-CD42-ABDF-55112CEEA85C}">
     <text>I'm fine.</text>
   </threadedComment>
+  <threadedComment ref="C4" dT="2026-07-07T06:59:34.40" personId="{3593DA02-0F55-9F40-9BF5-CE90CCFAECBC}" id="{7DB408AD-9FCB-6047-8FBF-78F298A51E18}">
+    <text>好的</text>
+  </threadedComment>
+  <threadedComment ref="C4" dT="2026-07-07T06:59:40.80" personId="{3593DA02-0F55-9F40-9BF5-CE90CCFAECBC}" id="{0BE16805-E50C-C645-B586-47F5D948E55A}" parentId="{7DB408AD-9FCB-6047-8FBF-78F298A51E18}">
+    <text>不错</text>
+  </threadedComment>
+  <threadedComment ref="C4" dT="2026-07-07T06:59:44.81" personId="{3593DA02-0F55-9F40-9BF5-CE90CCFAECBC}" id="{E0990B81-6C2E-7546-8FC1-3F7D23E5289F}" parentId="{7DB408AD-9FCB-6047-8FBF-78F298A51E18}">
+    <text>很好</text>
+  </threadedComment>
+  <threadedComment ref="C8" dT="2026-07-07T06:58:29.27" personId="{3593DA02-0F55-9F40-9BF5-CE90CCFAECBC}" id="{5139E8D2-ECA7-044F-8352-0F7F0BD80678}">
+    <text xml:space="preserve">world 
+</text>
+  </threadedComment>
+  <threadedComment ref="C8" dT="2026-07-07T06:58:40.92" personId="{3593DA02-0F55-9F40-9BF5-CE90CCFAECBC}" id="{AB927039-9B47-C34D-A3B5-F0B885B49F81}" parentId="{5139E8D2-ECA7-044F-8352-0F7F0BD80678}">
+    <text>这是回复</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FFAB8E1-8CEB-ED40-9EC3-FB8A667C0C67}">
-  <dimension ref="B2"/>
+  <dimension ref="B2:C8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:3">
       <c r="B2" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3">
+      <c r="C4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3">
+      <c r="C8" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>